<commit_message>
Update DateBase/orders/International Ever Green_2026-3-19.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/International Ever Green_2026-3-19.xlsx
+++ b/DateBase/orders/International Ever Green_2026-3-19.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,9 +488,62 @@
         <v>485_情人草_Limonium/Misty_undefined_1bunch</v>
       </c>
     </row>
+    <row r="12">
+      <c r="C12" t="str">
+        <v>486_水晶草_Limonium_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="str">
+        <v>594_绿毛球_undefined_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" t="str">
+        <v>383_油画向日葵_sunflower black_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="str">
+        <v>477_泰迪向日葵_sunflower Teddy_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" t="str">
+        <v>478_绿芯向日葵_sunflower mini_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="str">
+        <v>639_向日葵柠檬黄_undefined_undefined_1stem</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="str">
+        <v>577_腊梅白_wax white_undefined_1bunch</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="str">
+        <v>1_白洋桔梗_White Lisianthus_Eustoma grandiflorum (Raf.) Shinners_800/600g</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>2_粉洋桔梗_Pink Lisianthus_Eustoma grandiflorum (Raf.) Shinners_800/600g</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="str">
+        <v>3_波浪白洋桔梗_Wavy White Lisianthus_Eustoma grandiflorum (Raf.) Shinners_800/600g</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>